<commit_message>
Implement production line scheduling workflow
</commit_message>
<xml_diff>
--- a/backend/assets/零件导入模板.xlsx
+++ b/backend/assets/零件导入模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="零件导入" sheetId="1" r:id="Rcbe16f2181954f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rd2eb88523bfa4b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="零件导入" sheetId="1" r:id="R1e2bf3a96b8c4cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Re51c5d65bc3741fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -69,8 +69,18 @@
         <x:fgColor rgb="FFDDEFE8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0C4A3E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0C4A3E"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -137,11 +147,39 @@
         <x:color rgb="FFD7E3DE"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF0C4A3E"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF0C4A3E"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF0C4A3E"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF0C4A3E"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E3DE"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7E3DE"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7E3DE"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7E3DE"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +253,37 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -425,6 +494,7 @@
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -449,6 +519,9 @@
       <x:c r="G1" s="11" t="str">
         <x:v>员工2</x:v>
       </x:c>
+      <x:c r="H1" s="43" t="str">
+        <x:v>员工3</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="18"/>
@@ -458,6 +531,7 @@
       <x:c r="E2" s="16"/>
       <x:c r="F2" s="16"/>
       <x:c r="G2" s="16"/>
+      <x:c r="H2" s="42"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="19"/>
@@ -467,6 +541,7 @@
       <x:c r="E3" s="17"/>
       <x:c r="F3" s="17"/>
       <x:c r="G3" s="17"/>
+      <x:c r="H3" s="42"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="19"/>
@@ -476,6 +551,7 @@
       <x:c r="E4" s="17"/>
       <x:c r="F4" s="17"/>
       <x:c r="G4" s="17"/>
+      <x:c r="H4" s="42"/>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="19"/>
@@ -485,6 +561,7 @@
       <x:c r="E5" s="17"/>
       <x:c r="F5" s="17"/>
       <x:c r="G5" s="17"/>
+      <x:c r="H5" s="42"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="19"/>
@@ -494,6 +571,7 @@
       <x:c r="E6" s="17"/>
       <x:c r="F6" s="17"/>
       <x:c r="G6" s="17"/>
+      <x:c r="H6" s="42"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="19"/>
@@ -503,6 +581,7 @@
       <x:c r="E7" s="17"/>
       <x:c r="F7" s="17"/>
       <x:c r="G7" s="17"/>
+      <x:c r="H7" s="42"/>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="19"/>
@@ -512,6 +591,7 @@
       <x:c r="E8" s="17"/>
       <x:c r="F8" s="17"/>
       <x:c r="G8" s="17"/>
+      <x:c r="H8" s="42"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="19"/>
@@ -521,6 +601,7 @@
       <x:c r="E9" s="17"/>
       <x:c r="F9" s="17"/>
       <x:c r="G9" s="17"/>
+      <x:c r="H9" s="42"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="19"/>
@@ -530,6 +611,7 @@
       <x:c r="E10" s="17"/>
       <x:c r="F10" s="17"/>
       <x:c r="G10" s="17"/>
+      <x:c r="H10" s="42"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="19"/>
@@ -539,6 +621,7 @@
       <x:c r="E11" s="17"/>
       <x:c r="F11" s="17"/>
       <x:c r="G11" s="17"/>
+      <x:c r="H11" s="42"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="19"/>
@@ -548,6 +631,7 @@
       <x:c r="E12" s="17"/>
       <x:c r="F12" s="17"/>
       <x:c r="G12" s="17"/>
+      <x:c r="H12" s="42"/>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="19"/>
@@ -557,6 +641,7 @@
       <x:c r="E13" s="17"/>
       <x:c r="F13" s="17"/>
       <x:c r="G13" s="17"/>
+      <x:c r="H13" s="42"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="19"/>
@@ -566,6 +651,7 @@
       <x:c r="E14" s="17"/>
       <x:c r="F14" s="17"/>
       <x:c r="G14" s="17"/>
+      <x:c r="H14" s="42"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="19"/>
@@ -575,6 +661,7 @@
       <x:c r="E15" s="17"/>
       <x:c r="F15" s="17"/>
       <x:c r="G15" s="17"/>
+      <x:c r="H15" s="42"/>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="19"/>
@@ -584,6 +671,7 @@
       <x:c r="E16" s="17"/>
       <x:c r="F16" s="17"/>
       <x:c r="G16" s="17"/>
+      <x:c r="H16" s="42"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="19"/>
@@ -593,6 +681,7 @@
       <x:c r="E17" s="17"/>
       <x:c r="F17" s="17"/>
       <x:c r="G17" s="17"/>
+      <x:c r="H17" s="42"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="19"/>
@@ -602,6 +691,7 @@
       <x:c r="E18" s="17"/>
       <x:c r="F18" s="17"/>
       <x:c r="G18" s="17"/>
+      <x:c r="H18" s="42"/>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="19"/>
@@ -611,6 +701,7 @@
       <x:c r="E19" s="17"/>
       <x:c r="F19" s="17"/>
       <x:c r="G19" s="17"/>
+      <x:c r="H19" s="42"/>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="19"/>
@@ -620,6 +711,7 @@
       <x:c r="E20" s="17"/>
       <x:c r="F20" s="17"/>
       <x:c r="G20" s="17"/>
+      <x:c r="H20" s="42"/>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="19"/>
@@ -629,6 +721,7 @@
       <x:c r="E21" s="17"/>
       <x:c r="F21" s="17"/>
       <x:c r="G21" s="17"/>
+      <x:c r="H21" s="42"/>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="19"/>
@@ -638,6 +731,7 @@
       <x:c r="E22" s="17"/>
       <x:c r="F22" s="17"/>
       <x:c r="G22" s="17"/>
+      <x:c r="H22" s="42"/>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="19"/>
@@ -647,6 +741,7 @@
       <x:c r="E23" s="17"/>
       <x:c r="F23" s="17"/>
       <x:c r="G23" s="17"/>
+      <x:c r="H23" s="42"/>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="19"/>
@@ -656,6 +751,7 @@
       <x:c r="E24" s="17"/>
       <x:c r="F24" s="17"/>
       <x:c r="G24" s="17"/>
+      <x:c r="H24" s="42"/>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="19"/>
@@ -665,6 +761,7 @@
       <x:c r="E25" s="17"/>
       <x:c r="F25" s="17"/>
       <x:c r="G25" s="17"/>
+      <x:c r="H25" s="42"/>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="19"/>
@@ -674,6 +771,7 @@
       <x:c r="E26" s="17"/>
       <x:c r="F26" s="17"/>
       <x:c r="G26" s="17"/>
+      <x:c r="H26" s="42"/>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="19"/>
@@ -683,6 +781,7 @@
       <x:c r="E27" s="17"/>
       <x:c r="F27" s="17"/>
       <x:c r="G27" s="17"/>
+      <x:c r="H27" s="42"/>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="19"/>
@@ -692,6 +791,7 @@
       <x:c r="E28" s="17"/>
       <x:c r="F28" s="17"/>
       <x:c r="G28" s="17"/>
+      <x:c r="H28" s="42"/>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="19"/>
@@ -701,6 +801,7 @@
       <x:c r="E29" s="17"/>
       <x:c r="F29" s="17"/>
       <x:c r="G29" s="17"/>
+      <x:c r="H29" s="42"/>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="19"/>
@@ -710,6 +811,7 @@
       <x:c r="E30" s="17"/>
       <x:c r="F30" s="17"/>
       <x:c r="G30" s="17"/>
+      <x:c r="H30" s="42"/>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="19"/>
@@ -719,6 +821,7 @@
       <x:c r="E31" s="17"/>
       <x:c r="F31" s="17"/>
       <x:c r="G31" s="17"/>
+      <x:c r="H31" s="42"/>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="19"/>
@@ -728,6 +831,7 @@
       <x:c r="E32" s="17"/>
       <x:c r="F32" s="17"/>
       <x:c r="G32" s="17"/>
+      <x:c r="H32" s="42"/>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="19"/>
@@ -737,6 +841,7 @@
       <x:c r="E33" s="17"/>
       <x:c r="F33" s="17"/>
       <x:c r="G33" s="17"/>
+      <x:c r="H33" s="42"/>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="19"/>
@@ -746,6 +851,7 @@
       <x:c r="E34" s="17"/>
       <x:c r="F34" s="17"/>
       <x:c r="G34" s="17"/>
+      <x:c r="H34" s="42"/>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="19"/>
@@ -755,6 +861,7 @@
       <x:c r="E35" s="17"/>
       <x:c r="F35" s="17"/>
       <x:c r="G35" s="17"/>
+      <x:c r="H35" s="42"/>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="19"/>
@@ -764,6 +871,7 @@
       <x:c r="E36" s="17"/>
       <x:c r="F36" s="17"/>
       <x:c r="G36" s="17"/>
+      <x:c r="H36" s="42"/>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="19"/>
@@ -773,6 +881,7 @@
       <x:c r="E37" s="17"/>
       <x:c r="F37" s="17"/>
       <x:c r="G37" s="17"/>
+      <x:c r="H37" s="42"/>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="19"/>
@@ -782,6 +891,7 @@
       <x:c r="E38" s="17"/>
       <x:c r="F38" s="17"/>
       <x:c r="G38" s="17"/>
+      <x:c r="H38" s="42"/>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
       <x:c r="A39" s="19"/>
@@ -791,6 +901,7 @@
       <x:c r="E39" s="17"/>
       <x:c r="F39" s="17"/>
       <x:c r="G39" s="17"/>
+      <x:c r="H39" s="42"/>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="19"/>
@@ -800,6 +911,7 @@
       <x:c r="E40" s="17"/>
       <x:c r="F40" s="17"/>
       <x:c r="G40" s="17"/>
+      <x:c r="H40" s="42"/>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="19"/>
@@ -809,6 +921,7 @@
       <x:c r="E41" s="17"/>
       <x:c r="F41" s="17"/>
       <x:c r="G41" s="17"/>
+      <x:c r="H41" s="42"/>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="A42" s="19"/>
@@ -818,6 +931,7 @@
       <x:c r="E42" s="17"/>
       <x:c r="F42" s="17"/>
       <x:c r="G42" s="17"/>
+      <x:c r="H42" s="42"/>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="19"/>
@@ -827,6 +941,7 @@
       <x:c r="E43" s="17"/>
       <x:c r="F43" s="17"/>
       <x:c r="G43" s="17"/>
+      <x:c r="H43" s="42"/>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="19"/>
@@ -836,6 +951,7 @@
       <x:c r="E44" s="17"/>
       <x:c r="F44" s="17"/>
       <x:c r="G44" s="17"/>
+      <x:c r="H44" s="42"/>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
       <x:c r="A45" s="19"/>
@@ -845,6 +961,7 @@
       <x:c r="E45" s="17"/>
       <x:c r="F45" s="17"/>
       <x:c r="G45" s="17"/>
+      <x:c r="H45" s="42"/>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
       <x:c r="A46" s="19"/>
@@ -854,6 +971,7 @@
       <x:c r="E46" s="17"/>
       <x:c r="F46" s="17"/>
       <x:c r="G46" s="17"/>
+      <x:c r="H46" s="42"/>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
       <x:c r="A47" s="19"/>
@@ -863,6 +981,7 @@
       <x:c r="E47" s="17"/>
       <x:c r="F47" s="17"/>
       <x:c r="G47" s="17"/>
+      <x:c r="H47" s="42"/>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
       <x:c r="A48" s="19"/>
@@ -872,6 +991,7 @@
       <x:c r="E48" s="17"/>
       <x:c r="F48" s="17"/>
       <x:c r="G48" s="17"/>
+      <x:c r="H48" s="42"/>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
       <x:c r="A49" s="19"/>
@@ -881,6 +1001,7 @@
       <x:c r="E49" s="17"/>
       <x:c r="F49" s="17"/>
       <x:c r="G49" s="17"/>
+      <x:c r="H49" s="42"/>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
       <x:c r="A50" s="19"/>
@@ -890,6 +1011,7 @@
       <x:c r="E50" s="17"/>
       <x:c r="F50" s="17"/>
       <x:c r="G50" s="17"/>
+      <x:c r="H50" s="42"/>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
       <x:c r="A51" s="19"/>
@@ -899,6 +1021,7 @@
       <x:c r="E51" s="17"/>
       <x:c r="F51" s="17"/>
       <x:c r="G51" s="17"/>
+      <x:c r="H51" s="42"/>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
       <x:c r="A52" s="19"/>
@@ -908,6 +1031,7 @@
       <x:c r="E52" s="17"/>
       <x:c r="F52" s="17"/>
       <x:c r="G52" s="17"/>
+      <x:c r="H52" s="42"/>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
       <x:c r="A53" s="19"/>
@@ -917,6 +1041,7 @@
       <x:c r="E53" s="17"/>
       <x:c r="F53" s="17"/>
       <x:c r="G53" s="17"/>
+      <x:c r="H53" s="42"/>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
       <x:c r="A54" s="19"/>
@@ -926,6 +1051,7 @@
       <x:c r="E54" s="17"/>
       <x:c r="F54" s="17"/>
       <x:c r="G54" s="17"/>
+      <x:c r="H54" s="42"/>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
       <x:c r="A55" s="19"/>
@@ -935,6 +1061,7 @@
       <x:c r="E55" s="17"/>
       <x:c r="F55" s="17"/>
       <x:c r="G55" s="17"/>
+      <x:c r="H55" s="42"/>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
       <x:c r="A56" s="19"/>
@@ -944,6 +1071,7 @@
       <x:c r="E56" s="17"/>
       <x:c r="F56" s="17"/>
       <x:c r="G56" s="17"/>
+      <x:c r="H56" s="42"/>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
       <x:c r="A57" s="19"/>
@@ -953,6 +1081,7 @@
       <x:c r="E57" s="17"/>
       <x:c r="F57" s="17"/>
       <x:c r="G57" s="17"/>
+      <x:c r="H57" s="42"/>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
       <x:c r="A58" s="19"/>
@@ -962,6 +1091,7 @@
       <x:c r="E58" s="17"/>
       <x:c r="F58" s="17"/>
       <x:c r="G58" s="17"/>
+      <x:c r="H58" s="42"/>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
       <x:c r="A59" s="19"/>
@@ -971,6 +1101,7 @@
       <x:c r="E59" s="17"/>
       <x:c r="F59" s="17"/>
       <x:c r="G59" s="17"/>
+      <x:c r="H59" s="42"/>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
       <x:c r="A60" s="19"/>
@@ -980,6 +1111,7 @@
       <x:c r="E60" s="17"/>
       <x:c r="F60" s="17"/>
       <x:c r="G60" s="17"/>
+      <x:c r="H60" s="42"/>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
       <x:c r="A61" s="19"/>
@@ -989,6 +1121,7 @@
       <x:c r="E61" s="17"/>
       <x:c r="F61" s="17"/>
       <x:c r="G61" s="17"/>
+      <x:c r="H61" s="42"/>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
       <x:c r="A62" s="19"/>
@@ -998,6 +1131,7 @@
       <x:c r="E62" s="17"/>
       <x:c r="F62" s="17"/>
       <x:c r="G62" s="17"/>
+      <x:c r="H62" s="42"/>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
       <x:c r="A63" s="19"/>
@@ -1007,6 +1141,7 @@
       <x:c r="E63" s="17"/>
       <x:c r="F63" s="17"/>
       <x:c r="G63" s="17"/>
+      <x:c r="H63" s="42"/>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
       <x:c r="A64" s="19"/>
@@ -1016,6 +1151,7 @@
       <x:c r="E64" s="17"/>
       <x:c r="F64" s="17"/>
       <x:c r="G64" s="17"/>
+      <x:c r="H64" s="42"/>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
       <x:c r="A65" s="19"/>
@@ -1025,6 +1161,7 @@
       <x:c r="E65" s="17"/>
       <x:c r="F65" s="17"/>
       <x:c r="G65" s="17"/>
+      <x:c r="H65" s="42"/>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
       <x:c r="A66" s="19"/>
@@ -1034,6 +1171,7 @@
       <x:c r="E66" s="17"/>
       <x:c r="F66" s="17"/>
       <x:c r="G66" s="17"/>
+      <x:c r="H66" s="42"/>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
       <x:c r="A67" s="19"/>
@@ -1043,6 +1181,7 @@
       <x:c r="E67" s="17"/>
       <x:c r="F67" s="17"/>
       <x:c r="G67" s="17"/>
+      <x:c r="H67" s="42"/>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
       <x:c r="A68" s="19"/>
@@ -1052,6 +1191,7 @@
       <x:c r="E68" s="17"/>
       <x:c r="F68" s="17"/>
       <x:c r="G68" s="17"/>
+      <x:c r="H68" s="42"/>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
       <x:c r="A69" s="19"/>
@@ -1061,6 +1201,7 @@
       <x:c r="E69" s="17"/>
       <x:c r="F69" s="17"/>
       <x:c r="G69" s="17"/>
+      <x:c r="H69" s="42"/>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
       <x:c r="A70" s="19"/>
@@ -1070,6 +1211,7 @@
       <x:c r="E70" s="17"/>
       <x:c r="F70" s="17"/>
       <x:c r="G70" s="17"/>
+      <x:c r="H70" s="42"/>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
       <x:c r="A71" s="19"/>
@@ -1079,6 +1221,7 @@
       <x:c r="E71" s="17"/>
       <x:c r="F71" s="17"/>
       <x:c r="G71" s="17"/>
+      <x:c r="H71" s="42"/>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
       <x:c r="A72" s="19"/>
@@ -1088,6 +1231,7 @@
       <x:c r="E72" s="17"/>
       <x:c r="F72" s="17"/>
       <x:c r="G72" s="17"/>
+      <x:c r="H72" s="42"/>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
       <x:c r="A73" s="19"/>
@@ -1097,6 +1241,7 @@
       <x:c r="E73" s="17"/>
       <x:c r="F73" s="17"/>
       <x:c r="G73" s="17"/>
+      <x:c r="H73" s="42"/>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
       <x:c r="A74" s="19"/>
@@ -1106,6 +1251,7 @@
       <x:c r="E74" s="17"/>
       <x:c r="F74" s="17"/>
       <x:c r="G74" s="17"/>
+      <x:c r="H74" s="42"/>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
       <x:c r="A75" s="19"/>
@@ -1115,6 +1261,7 @@
       <x:c r="E75" s="17"/>
       <x:c r="F75" s="17"/>
       <x:c r="G75" s="17"/>
+      <x:c r="H75" s="42"/>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
       <x:c r="A76" s="19"/>
@@ -1124,6 +1271,7 @@
       <x:c r="E76" s="17"/>
       <x:c r="F76" s="17"/>
       <x:c r="G76" s="17"/>
+      <x:c r="H76" s="42"/>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
       <x:c r="A77" s="19"/>
@@ -1133,6 +1281,7 @@
       <x:c r="E77" s="17"/>
       <x:c r="F77" s="17"/>
       <x:c r="G77" s="17"/>
+      <x:c r="H77" s="42"/>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
       <x:c r="A78" s="19"/>
@@ -1142,6 +1291,7 @@
       <x:c r="E78" s="17"/>
       <x:c r="F78" s="17"/>
       <x:c r="G78" s="17"/>
+      <x:c r="H78" s="42"/>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
       <x:c r="A79" s="19"/>
@@ -1151,6 +1301,7 @@
       <x:c r="E79" s="17"/>
       <x:c r="F79" s="17"/>
       <x:c r="G79" s="17"/>
+      <x:c r="H79" s="42"/>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
       <x:c r="A80" s="19"/>
@@ -1160,6 +1311,7 @@
       <x:c r="E80" s="17"/>
       <x:c r="F80" s="17"/>
       <x:c r="G80" s="17"/>
+      <x:c r="H80" s="42"/>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
       <x:c r="A81" s="19"/>
@@ -1169,6 +1321,7 @@
       <x:c r="E81" s="17"/>
       <x:c r="F81" s="17"/>
       <x:c r="G81" s="17"/>
+      <x:c r="H81" s="42"/>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
       <x:c r="A82" s="19"/>
@@ -1178,6 +1331,7 @@
       <x:c r="E82" s="17"/>
       <x:c r="F82" s="17"/>
       <x:c r="G82" s="17"/>
+      <x:c r="H82" s="42"/>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
       <x:c r="A83" s="19"/>
@@ -1187,6 +1341,7 @@
       <x:c r="E83" s="17"/>
       <x:c r="F83" s="17"/>
       <x:c r="G83" s="17"/>
+      <x:c r="H83" s="42"/>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
       <x:c r="A84" s="19"/>
@@ -1196,6 +1351,7 @@
       <x:c r="E84" s="17"/>
       <x:c r="F84" s="17"/>
       <x:c r="G84" s="17"/>
+      <x:c r="H84" s="42"/>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
       <x:c r="A85" s="19"/>
@@ -1205,6 +1361,7 @@
       <x:c r="E85" s="17"/>
       <x:c r="F85" s="17"/>
       <x:c r="G85" s="17"/>
+      <x:c r="H85" s="42"/>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
       <x:c r="A86" s="19"/>
@@ -1214,6 +1371,7 @@
       <x:c r="E86" s="17"/>
       <x:c r="F86" s="17"/>
       <x:c r="G86" s="17"/>
+      <x:c r="H86" s="42"/>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
       <x:c r="A87" s="19"/>
@@ -1223,6 +1381,7 @@
       <x:c r="E87" s="17"/>
       <x:c r="F87" s="17"/>
       <x:c r="G87" s="17"/>
+      <x:c r="H87" s="42"/>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
       <x:c r="A88" s="19"/>
@@ -1232,6 +1391,7 @@
       <x:c r="E88" s="17"/>
       <x:c r="F88" s="17"/>
       <x:c r="G88" s="17"/>
+      <x:c r="H88" s="42"/>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
       <x:c r="A89" s="19"/>
@@ -1241,6 +1401,7 @@
       <x:c r="E89" s="17"/>
       <x:c r="F89" s="17"/>
       <x:c r="G89" s="17"/>
+      <x:c r="H89" s="42"/>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
       <x:c r="A90" s="19"/>
@@ -1250,6 +1411,7 @@
       <x:c r="E90" s="17"/>
       <x:c r="F90" s="17"/>
       <x:c r="G90" s="17"/>
+      <x:c r="H90" s="42"/>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
       <x:c r="A91" s="19"/>
@@ -1259,6 +1421,7 @@
       <x:c r="E91" s="17"/>
       <x:c r="F91" s="17"/>
       <x:c r="G91" s="17"/>
+      <x:c r="H91" s="42"/>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
       <x:c r="A92" s="19"/>
@@ -1268,6 +1431,7 @@
       <x:c r="E92" s="17"/>
       <x:c r="F92" s="17"/>
       <x:c r="G92" s="17"/>
+      <x:c r="H92" s="42"/>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
       <x:c r="A93" s="19"/>
@@ -1277,6 +1441,7 @@
       <x:c r="E93" s="17"/>
       <x:c r="F93" s="17"/>
       <x:c r="G93" s="17"/>
+      <x:c r="H93" s="42"/>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
       <x:c r="A94" s="19"/>
@@ -1286,6 +1451,7 @@
       <x:c r="E94" s="17"/>
       <x:c r="F94" s="17"/>
       <x:c r="G94" s="17"/>
+      <x:c r="H94" s="42"/>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
       <x:c r="A95" s="19"/>
@@ -1295,6 +1461,7 @@
       <x:c r="E95" s="17"/>
       <x:c r="F95" s="17"/>
       <x:c r="G95" s="17"/>
+      <x:c r="H95" s="42"/>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
       <x:c r="A96" s="19"/>
@@ -1304,6 +1471,7 @@
       <x:c r="E96" s="17"/>
       <x:c r="F96" s="17"/>
       <x:c r="G96" s="17"/>
+      <x:c r="H96" s="42"/>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
       <x:c r="A97" s="19"/>
@@ -1313,6 +1481,7 @@
       <x:c r="E97" s="17"/>
       <x:c r="F97" s="17"/>
       <x:c r="G97" s="17"/>
+      <x:c r="H97" s="42"/>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
       <x:c r="A98" s="19"/>
@@ -1322,6 +1491,7 @@
       <x:c r="E98" s="17"/>
       <x:c r="F98" s="17"/>
       <x:c r="G98" s="17"/>
+      <x:c r="H98" s="42"/>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
       <x:c r="A99" s="19"/>
@@ -1331,6 +1501,7 @@
       <x:c r="E99" s="17"/>
       <x:c r="F99" s="17"/>
       <x:c r="G99" s="17"/>
+      <x:c r="H99" s="42"/>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
       <x:c r="A100" s="19"/>
@@ -1340,6 +1511,7 @@
       <x:c r="E100" s="17"/>
       <x:c r="F100" s="17"/>
       <x:c r="G100" s="17"/>
+      <x:c r="H100" s="42"/>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
       <x:c r="A101" s="19"/>
@@ -1349,6 +1521,7 @@
       <x:c r="E101" s="17"/>
       <x:c r="F101" s="17"/>
       <x:c r="G101" s="17"/>
+      <x:c r="H101" s="42"/>
     </x:row>
     <x:row r="102" ht="24" customHeight="1">
       <x:c r="A102" s="19"/>
@@ -1358,6 +1531,7 @@
       <x:c r="E102" s="17"/>
       <x:c r="F102" s="17"/>
       <x:c r="G102" s="17"/>
+      <x:c r="H102" s="42"/>
     </x:row>
     <x:row r="103" ht="24" customHeight="1">
       <x:c r="A103" s="19"/>
@@ -1367,6 +1541,7 @@
       <x:c r="E103" s="17"/>
       <x:c r="F103" s="17"/>
       <x:c r="G103" s="17"/>
+      <x:c r="H103" s="42"/>
     </x:row>
     <x:row r="104" ht="24" customHeight="1">
       <x:c r="A104" s="19"/>
@@ -1376,6 +1551,7 @@
       <x:c r="E104" s="17"/>
       <x:c r="F104" s="17"/>
       <x:c r="G104" s="17"/>
+      <x:c r="H104" s="42"/>
     </x:row>
     <x:row r="105" ht="24" customHeight="1">
       <x:c r="A105" s="19"/>
@@ -1385,6 +1561,7 @@
       <x:c r="E105" s="17"/>
       <x:c r="F105" s="17"/>
       <x:c r="G105" s="17"/>
+      <x:c r="H105" s="42"/>
     </x:row>
     <x:row r="106" ht="24" customHeight="1">
       <x:c r="A106" s="19"/>
@@ -1394,6 +1571,7 @@
       <x:c r="E106" s="17"/>
       <x:c r="F106" s="17"/>
       <x:c r="G106" s="17"/>
+      <x:c r="H106" s="42"/>
     </x:row>
     <x:row r="107" ht="24" customHeight="1">
       <x:c r="A107" s="19"/>
@@ -1403,6 +1581,7 @@
       <x:c r="E107" s="17"/>
       <x:c r="F107" s="17"/>
       <x:c r="G107" s="17"/>
+      <x:c r="H107" s="42"/>
     </x:row>
     <x:row r="108" ht="24" customHeight="1">
       <x:c r="A108" s="19"/>
@@ -1412,6 +1591,7 @@
       <x:c r="E108" s="17"/>
       <x:c r="F108" s="17"/>
       <x:c r="G108" s="17"/>
+      <x:c r="H108" s="42"/>
     </x:row>
     <x:row r="109" ht="24" customHeight="1">
       <x:c r="A109" s="19"/>
@@ -1421,6 +1601,7 @@
       <x:c r="E109" s="17"/>
       <x:c r="F109" s="17"/>
       <x:c r="G109" s="17"/>
+      <x:c r="H109" s="42"/>
     </x:row>
     <x:row r="110" ht="24" customHeight="1">
       <x:c r="A110" s="19"/>
@@ -1430,6 +1611,7 @@
       <x:c r="E110" s="17"/>
       <x:c r="F110" s="17"/>
       <x:c r="G110" s="17"/>
+      <x:c r="H110" s="42"/>
     </x:row>
     <x:row r="111" ht="24" customHeight="1">
       <x:c r="A111" s="19"/>
@@ -1439,6 +1621,7 @@
       <x:c r="E111" s="17"/>
       <x:c r="F111" s="17"/>
       <x:c r="G111" s="17"/>
+      <x:c r="H111" s="42"/>
     </x:row>
     <x:row r="112" ht="24" customHeight="1">
       <x:c r="A112" s="19"/>
@@ -1448,6 +1631,7 @@
       <x:c r="E112" s="17"/>
       <x:c r="F112" s="17"/>
       <x:c r="G112" s="17"/>
+      <x:c r="H112" s="42"/>
     </x:row>
     <x:row r="113" ht="24" customHeight="1">
       <x:c r="A113" s="19"/>
@@ -1457,6 +1641,7 @@
       <x:c r="E113" s="17"/>
       <x:c r="F113" s="17"/>
       <x:c r="G113" s="17"/>
+      <x:c r="H113" s="42"/>
     </x:row>
     <x:row r="114" ht="24" customHeight="1">
       <x:c r="A114" s="19"/>
@@ -1466,6 +1651,7 @@
       <x:c r="E114" s="17"/>
       <x:c r="F114" s="17"/>
       <x:c r="G114" s="17"/>
+      <x:c r="H114" s="42"/>
     </x:row>
     <x:row r="115" ht="24" customHeight="1">
       <x:c r="A115" s="19"/>
@@ -1475,6 +1661,7 @@
       <x:c r="E115" s="17"/>
       <x:c r="F115" s="17"/>
       <x:c r="G115" s="17"/>
+      <x:c r="H115" s="42"/>
     </x:row>
     <x:row r="116" ht="24" customHeight="1">
       <x:c r="A116" s="19"/>
@@ -1484,6 +1671,7 @@
       <x:c r="E116" s="17"/>
       <x:c r="F116" s="17"/>
       <x:c r="G116" s="17"/>
+      <x:c r="H116" s="42"/>
     </x:row>
     <x:row r="117" ht="24" customHeight="1">
       <x:c r="A117" s="19"/>
@@ -1493,6 +1681,7 @@
       <x:c r="E117" s="17"/>
       <x:c r="F117" s="17"/>
       <x:c r="G117" s="17"/>
+      <x:c r="H117" s="42"/>
     </x:row>
     <x:row r="118" ht="24" customHeight="1">
       <x:c r="A118" s="19"/>
@@ -1502,6 +1691,7 @@
       <x:c r="E118" s="17"/>
       <x:c r="F118" s="17"/>
       <x:c r="G118" s="17"/>
+      <x:c r="H118" s="42"/>
     </x:row>
     <x:row r="119" ht="24" customHeight="1">
       <x:c r="A119" s="19"/>
@@ -1511,6 +1701,7 @@
       <x:c r="E119" s="17"/>
       <x:c r="F119" s="17"/>
       <x:c r="G119" s="17"/>
+      <x:c r="H119" s="42"/>
     </x:row>
     <x:row r="120" ht="24" customHeight="1">
       <x:c r="A120" s="19"/>
@@ -1520,6 +1711,7 @@
       <x:c r="E120" s="17"/>
       <x:c r="F120" s="17"/>
       <x:c r="G120" s="17"/>
+      <x:c r="H120" s="42"/>
     </x:row>
     <x:row r="121" ht="24" customHeight="1">
       <x:c r="A121" s="19"/>
@@ -1529,6 +1721,7 @@
       <x:c r="E121" s="17"/>
       <x:c r="F121" s="17"/>
       <x:c r="G121" s="17"/>
+      <x:c r="H121" s="42"/>
     </x:row>
     <x:row r="122" ht="24" customHeight="1">
       <x:c r="A122" s="19"/>
@@ -1538,6 +1731,7 @@
       <x:c r="E122" s="17"/>
       <x:c r="F122" s="17"/>
       <x:c r="G122" s="17"/>
+      <x:c r="H122" s="42"/>
     </x:row>
     <x:row r="123" ht="24" customHeight="1">
       <x:c r="A123" s="19"/>
@@ -1547,6 +1741,7 @@
       <x:c r="E123" s="17"/>
       <x:c r="F123" s="17"/>
       <x:c r="G123" s="17"/>
+      <x:c r="H123" s="42"/>
     </x:row>
     <x:row r="124" ht="24" customHeight="1">
       <x:c r="A124" s="19"/>
@@ -1556,6 +1751,7 @@
       <x:c r="E124" s="17"/>
       <x:c r="F124" s="17"/>
       <x:c r="G124" s="17"/>
+      <x:c r="H124" s="42"/>
     </x:row>
     <x:row r="125" ht="24" customHeight="1">
       <x:c r="A125" s="19"/>
@@ -1565,6 +1761,7 @@
       <x:c r="E125" s="17"/>
       <x:c r="F125" s="17"/>
       <x:c r="G125" s="17"/>
+      <x:c r="H125" s="42"/>
     </x:row>
     <x:row r="126" ht="24" customHeight="1">
       <x:c r="A126" s="19"/>
@@ -1574,6 +1771,7 @@
       <x:c r="E126" s="17"/>
       <x:c r="F126" s="17"/>
       <x:c r="G126" s="17"/>
+      <x:c r="H126" s="42"/>
     </x:row>
     <x:row r="127" ht="24" customHeight="1">
       <x:c r="A127" s="19"/>
@@ -1583,6 +1781,7 @@
       <x:c r="E127" s="17"/>
       <x:c r="F127" s="17"/>
       <x:c r="G127" s="17"/>
+      <x:c r="H127" s="42"/>
     </x:row>
     <x:row r="128" ht="24" customHeight="1">
       <x:c r="A128" s="19"/>
@@ -1592,6 +1791,7 @@
       <x:c r="E128" s="17"/>
       <x:c r="F128" s="17"/>
       <x:c r="G128" s="17"/>
+      <x:c r="H128" s="42"/>
     </x:row>
     <x:row r="129" ht="24" customHeight="1">
       <x:c r="A129" s="19"/>
@@ -1601,6 +1801,7 @@
       <x:c r="E129" s="17"/>
       <x:c r="F129" s="17"/>
       <x:c r="G129" s="17"/>
+      <x:c r="H129" s="42"/>
     </x:row>
     <x:row r="130" ht="24" customHeight="1">
       <x:c r="A130" s="19"/>
@@ -1610,6 +1811,7 @@
       <x:c r="E130" s="17"/>
       <x:c r="F130" s="17"/>
       <x:c r="G130" s="17"/>
+      <x:c r="H130" s="42"/>
     </x:row>
     <x:row r="131" ht="24" customHeight="1">
       <x:c r="A131" s="19"/>
@@ -1619,6 +1821,7 @@
       <x:c r="E131" s="17"/>
       <x:c r="F131" s="17"/>
       <x:c r="G131" s="17"/>
+      <x:c r="H131" s="42"/>
     </x:row>
     <x:row r="132" ht="24" customHeight="1">
       <x:c r="A132" s="19"/>
@@ -1628,6 +1831,7 @@
       <x:c r="E132" s="17"/>
       <x:c r="F132" s="17"/>
       <x:c r="G132" s="17"/>
+      <x:c r="H132" s="42"/>
     </x:row>
     <x:row r="133" ht="24" customHeight="1">
       <x:c r="A133" s="19"/>
@@ -1637,6 +1841,7 @@
       <x:c r="E133" s="17"/>
       <x:c r="F133" s="17"/>
       <x:c r="G133" s="17"/>
+      <x:c r="H133" s="42"/>
     </x:row>
     <x:row r="134" ht="24" customHeight="1">
       <x:c r="A134" s="19"/>
@@ -1646,6 +1851,7 @@
       <x:c r="E134" s="17"/>
       <x:c r="F134" s="17"/>
       <x:c r="G134" s="17"/>
+      <x:c r="H134" s="42"/>
     </x:row>
     <x:row r="135" ht="24" customHeight="1">
       <x:c r="A135" s="19"/>
@@ -1655,6 +1861,7 @@
       <x:c r="E135" s="17"/>
       <x:c r="F135" s="17"/>
       <x:c r="G135" s="17"/>
+      <x:c r="H135" s="42"/>
     </x:row>
     <x:row r="136" ht="24" customHeight="1">
       <x:c r="A136" s="19"/>
@@ -1664,6 +1871,7 @@
       <x:c r="E136" s="17"/>
       <x:c r="F136" s="17"/>
       <x:c r="G136" s="17"/>
+      <x:c r="H136" s="42"/>
     </x:row>
     <x:row r="137" ht="24" customHeight="1">
       <x:c r="A137" s="19"/>
@@ -1673,6 +1881,7 @@
       <x:c r="E137" s="17"/>
       <x:c r="F137" s="17"/>
       <x:c r="G137" s="17"/>
+      <x:c r="H137" s="42"/>
     </x:row>
     <x:row r="138" ht="24" customHeight="1">
       <x:c r="A138" s="19"/>
@@ -1682,6 +1891,7 @@
       <x:c r="E138" s="17"/>
       <x:c r="F138" s="17"/>
       <x:c r="G138" s="17"/>
+      <x:c r="H138" s="42"/>
     </x:row>
     <x:row r="139" ht="24" customHeight="1">
       <x:c r="A139" s="19"/>
@@ -1691,6 +1901,7 @@
       <x:c r="E139" s="17"/>
       <x:c r="F139" s="17"/>
       <x:c r="G139" s="17"/>
+      <x:c r="H139" s="42"/>
     </x:row>
     <x:row r="140" ht="24" customHeight="1">
       <x:c r="A140" s="19"/>
@@ -1700,6 +1911,7 @@
       <x:c r="E140" s="17"/>
       <x:c r="F140" s="17"/>
       <x:c r="G140" s="17"/>
+      <x:c r="H140" s="42"/>
     </x:row>
     <x:row r="141" ht="24" customHeight="1">
       <x:c r="A141" s="19"/>
@@ -1709,6 +1921,7 @@
       <x:c r="E141" s="17"/>
       <x:c r="F141" s="17"/>
       <x:c r="G141" s="17"/>
+      <x:c r="H141" s="42"/>
     </x:row>
     <x:row r="142" ht="24" customHeight="1">
       <x:c r="A142" s="19"/>
@@ -1718,6 +1931,7 @@
       <x:c r="E142" s="17"/>
       <x:c r="F142" s="17"/>
       <x:c r="G142" s="17"/>
+      <x:c r="H142" s="42"/>
     </x:row>
     <x:row r="143" ht="24" customHeight="1">
       <x:c r="A143" s="19"/>
@@ -1727,6 +1941,7 @@
       <x:c r="E143" s="17"/>
       <x:c r="F143" s="17"/>
       <x:c r="G143" s="17"/>
+      <x:c r="H143" s="42"/>
     </x:row>
     <x:row r="144" ht="24" customHeight="1">
       <x:c r="A144" s="19"/>
@@ -1736,6 +1951,7 @@
       <x:c r="E144" s="17"/>
       <x:c r="F144" s="17"/>
       <x:c r="G144" s="17"/>
+      <x:c r="H144" s="42"/>
     </x:row>
     <x:row r="145" ht="24" customHeight="1">
       <x:c r="A145" s="19"/>
@@ -1745,6 +1961,7 @@
       <x:c r="E145" s="17"/>
       <x:c r="F145" s="17"/>
       <x:c r="G145" s="17"/>
+      <x:c r="H145" s="42"/>
     </x:row>
     <x:row r="146" ht="24" customHeight="1">
       <x:c r="A146" s="19"/>
@@ -1754,6 +1971,7 @@
       <x:c r="E146" s="17"/>
       <x:c r="F146" s="17"/>
       <x:c r="G146" s="17"/>
+      <x:c r="H146" s="42"/>
     </x:row>
     <x:row r="147" ht="24" customHeight="1">
       <x:c r="A147" s="19"/>
@@ -1763,6 +1981,7 @@
       <x:c r="E147" s="17"/>
       <x:c r="F147" s="17"/>
       <x:c r="G147" s="17"/>
+      <x:c r="H147" s="42"/>
     </x:row>
     <x:row r="148" ht="24" customHeight="1">
       <x:c r="A148" s="19"/>
@@ -1772,6 +1991,7 @@
       <x:c r="E148" s="17"/>
       <x:c r="F148" s="17"/>
       <x:c r="G148" s="17"/>
+      <x:c r="H148" s="42"/>
     </x:row>
     <x:row r="149" ht="24" customHeight="1">
       <x:c r="A149" s="19"/>
@@ -1781,6 +2001,7 @@
       <x:c r="E149" s="17"/>
       <x:c r="F149" s="17"/>
       <x:c r="G149" s="17"/>
+      <x:c r="H149" s="42"/>
     </x:row>
     <x:row r="150" ht="24" customHeight="1">
       <x:c r="A150" s="19"/>
@@ -1790,6 +2011,7 @@
       <x:c r="E150" s="17"/>
       <x:c r="F150" s="17"/>
       <x:c r="G150" s="17"/>
+      <x:c r="H150" s="42"/>
     </x:row>
     <x:row r="151" ht="24" customHeight="1">
       <x:c r="A151" s="19"/>
@@ -1799,6 +2021,7 @@
       <x:c r="E151" s="17"/>
       <x:c r="F151" s="17"/>
       <x:c r="G151" s="17"/>
+      <x:c r="H151" s="42"/>
     </x:row>
     <x:row r="152" ht="24" customHeight="1">
       <x:c r="A152" s="19"/>
@@ -1808,6 +2031,7 @@
       <x:c r="E152" s="17"/>
       <x:c r="F152" s="17"/>
       <x:c r="G152" s="17"/>
+      <x:c r="H152" s="42"/>
     </x:row>
     <x:row r="153" ht="24" customHeight="1">
       <x:c r="A153" s="19"/>
@@ -1817,6 +2041,7 @@
       <x:c r="E153" s="17"/>
       <x:c r="F153" s="17"/>
       <x:c r="G153" s="17"/>
+      <x:c r="H153" s="42"/>
     </x:row>
     <x:row r="154" ht="24" customHeight="1">
       <x:c r="A154" s="19"/>
@@ -1826,6 +2051,7 @@
       <x:c r="E154" s="17"/>
       <x:c r="F154" s="17"/>
       <x:c r="G154" s="17"/>
+      <x:c r="H154" s="42"/>
     </x:row>
     <x:row r="155" ht="24" customHeight="1">
       <x:c r="A155" s="19"/>
@@ -1835,6 +2061,7 @@
       <x:c r="E155" s="17"/>
       <x:c r="F155" s="17"/>
       <x:c r="G155" s="17"/>
+      <x:c r="H155" s="42"/>
     </x:row>
     <x:row r="156" ht="24" customHeight="1">
       <x:c r="A156" s="19"/>
@@ -1844,6 +2071,7 @@
       <x:c r="E156" s="17"/>
       <x:c r="F156" s="17"/>
       <x:c r="G156" s="17"/>
+      <x:c r="H156" s="42"/>
     </x:row>
     <x:row r="157" ht="24" customHeight="1">
       <x:c r="A157" s="19"/>
@@ -1853,6 +2081,7 @@
       <x:c r="E157" s="17"/>
       <x:c r="F157" s="17"/>
       <x:c r="G157" s="17"/>
+      <x:c r="H157" s="42"/>
     </x:row>
     <x:row r="158" ht="24" customHeight="1">
       <x:c r="A158" s="19"/>
@@ -1862,6 +2091,7 @@
       <x:c r="E158" s="17"/>
       <x:c r="F158" s="17"/>
       <x:c r="G158" s="17"/>
+      <x:c r="H158" s="42"/>
     </x:row>
     <x:row r="159" ht="24" customHeight="1">
       <x:c r="A159" s="19"/>
@@ -1871,6 +2101,7 @@
       <x:c r="E159" s="17"/>
       <x:c r="F159" s="17"/>
       <x:c r="G159" s="17"/>
+      <x:c r="H159" s="42"/>
     </x:row>
     <x:row r="160" ht="24" customHeight="1">
       <x:c r="A160" s="19"/>
@@ -1880,6 +2111,7 @@
       <x:c r="E160" s="17"/>
       <x:c r="F160" s="17"/>
       <x:c r="G160" s="17"/>
+      <x:c r="H160" s="42"/>
     </x:row>
     <x:row r="161" ht="24" customHeight="1">
       <x:c r="A161" s="19"/>
@@ -1889,6 +2121,7 @@
       <x:c r="E161" s="17"/>
       <x:c r="F161" s="17"/>
       <x:c r="G161" s="17"/>
+      <x:c r="H161" s="42"/>
     </x:row>
     <x:row r="162" ht="24" customHeight="1">
       <x:c r="A162" s="19"/>
@@ -1898,6 +2131,7 @@
       <x:c r="E162" s="17"/>
       <x:c r="F162" s="17"/>
       <x:c r="G162" s="17"/>
+      <x:c r="H162" s="42"/>
     </x:row>
     <x:row r="163" ht="24" customHeight="1">
       <x:c r="A163" s="19"/>
@@ -1907,6 +2141,7 @@
       <x:c r="E163" s="17"/>
       <x:c r="F163" s="17"/>
       <x:c r="G163" s="17"/>
+      <x:c r="H163" s="42"/>
     </x:row>
     <x:row r="164" ht="24" customHeight="1">
       <x:c r="A164" s="19"/>
@@ -1916,6 +2151,7 @@
       <x:c r="E164" s="17"/>
       <x:c r="F164" s="17"/>
       <x:c r="G164" s="17"/>
+      <x:c r="H164" s="42"/>
     </x:row>
     <x:row r="165" ht="24" customHeight="1">
       <x:c r="A165" s="19"/>
@@ -1925,6 +2161,7 @@
       <x:c r="E165" s="17"/>
       <x:c r="F165" s="17"/>
       <x:c r="G165" s="17"/>
+      <x:c r="H165" s="42"/>
     </x:row>
     <x:row r="166" ht="24" customHeight="1">
       <x:c r="A166" s="19"/>
@@ -1934,6 +2171,7 @@
       <x:c r="E166" s="17"/>
       <x:c r="F166" s="17"/>
       <x:c r="G166" s="17"/>
+      <x:c r="H166" s="42"/>
     </x:row>
     <x:row r="167" ht="24" customHeight="1">
       <x:c r="A167" s="19"/>
@@ -1943,6 +2181,7 @@
       <x:c r="E167" s="17"/>
       <x:c r="F167" s="17"/>
       <x:c r="G167" s="17"/>
+      <x:c r="H167" s="42"/>
     </x:row>
     <x:row r="168" ht="24" customHeight="1">
       <x:c r="A168" s="19"/>
@@ -1952,6 +2191,7 @@
       <x:c r="E168" s="17"/>
       <x:c r="F168" s="17"/>
       <x:c r="G168" s="17"/>
+      <x:c r="H168" s="42"/>
     </x:row>
     <x:row r="169" ht="24" customHeight="1">
       <x:c r="A169" s="19"/>
@@ -1961,6 +2201,7 @@
       <x:c r="E169" s="17"/>
       <x:c r="F169" s="17"/>
       <x:c r="G169" s="17"/>
+      <x:c r="H169" s="42"/>
     </x:row>
     <x:row r="170" ht="24" customHeight="1">
       <x:c r="A170" s="19"/>
@@ -1970,6 +2211,7 @@
       <x:c r="E170" s="17"/>
       <x:c r="F170" s="17"/>
       <x:c r="G170" s="17"/>
+      <x:c r="H170" s="42"/>
     </x:row>
     <x:row r="171" ht="24" customHeight="1">
       <x:c r="A171" s="19"/>
@@ -1979,6 +2221,7 @@
       <x:c r="E171" s="17"/>
       <x:c r="F171" s="17"/>
       <x:c r="G171" s="17"/>
+      <x:c r="H171" s="42"/>
     </x:row>
     <x:row r="172" ht="24" customHeight="1">
       <x:c r="A172" s="19"/>
@@ -1988,6 +2231,7 @@
       <x:c r="E172" s="17"/>
       <x:c r="F172" s="17"/>
       <x:c r="G172" s="17"/>
+      <x:c r="H172" s="42"/>
     </x:row>
     <x:row r="173" ht="24" customHeight="1">
       <x:c r="A173" s="19"/>
@@ -1997,6 +2241,7 @@
       <x:c r="E173" s="17"/>
       <x:c r="F173" s="17"/>
       <x:c r="G173" s="17"/>
+      <x:c r="H173" s="42"/>
     </x:row>
     <x:row r="174" ht="24" customHeight="1">
       <x:c r="A174" s="19"/>
@@ -2006,6 +2251,7 @@
       <x:c r="E174" s="17"/>
       <x:c r="F174" s="17"/>
       <x:c r="G174" s="17"/>
+      <x:c r="H174" s="42"/>
     </x:row>
     <x:row r="175" ht="24" customHeight="1">
       <x:c r="A175" s="19"/>
@@ -2015,6 +2261,7 @@
       <x:c r="E175" s="17"/>
       <x:c r="F175" s="17"/>
       <x:c r="G175" s="17"/>
+      <x:c r="H175" s="42"/>
     </x:row>
     <x:row r="176" ht="24" customHeight="1">
       <x:c r="A176" s="19"/>
@@ -2024,6 +2271,7 @@
       <x:c r="E176" s="17"/>
       <x:c r="F176" s="17"/>
       <x:c r="G176" s="17"/>
+      <x:c r="H176" s="42"/>
     </x:row>
     <x:row r="177" ht="24" customHeight="1">
       <x:c r="A177" s="19"/>
@@ -2033,6 +2281,7 @@
       <x:c r="E177" s="17"/>
       <x:c r="F177" s="17"/>
       <x:c r="G177" s="17"/>
+      <x:c r="H177" s="42"/>
     </x:row>
     <x:row r="178" ht="24" customHeight="1">
       <x:c r="A178" s="19"/>
@@ -2042,6 +2291,7 @@
       <x:c r="E178" s="17"/>
       <x:c r="F178" s="17"/>
       <x:c r="G178" s="17"/>
+      <x:c r="H178" s="42"/>
     </x:row>
     <x:row r="179" ht="24" customHeight="1">
       <x:c r="A179" s="19"/>
@@ -2051,6 +2301,7 @@
       <x:c r="E179" s="17"/>
       <x:c r="F179" s="17"/>
       <x:c r="G179" s="17"/>
+      <x:c r="H179" s="42"/>
     </x:row>
     <x:row r="180" ht="24" customHeight="1">
       <x:c r="A180" s="19"/>
@@ -2060,6 +2311,7 @@
       <x:c r="E180" s="17"/>
       <x:c r="F180" s="17"/>
       <x:c r="G180" s="17"/>
+      <x:c r="H180" s="42"/>
     </x:row>
     <x:row r="181" ht="24" customHeight="1">
       <x:c r="A181" s="19"/>
@@ -2069,6 +2321,7 @@
       <x:c r="E181" s="17"/>
       <x:c r="F181" s="17"/>
       <x:c r="G181" s="17"/>
+      <x:c r="H181" s="42"/>
     </x:row>
     <x:row r="182" ht="24" customHeight="1">
       <x:c r="A182" s="19"/>
@@ -2078,6 +2331,7 @@
       <x:c r="E182" s="17"/>
       <x:c r="F182" s="17"/>
       <x:c r="G182" s="17"/>
+      <x:c r="H182" s="42"/>
     </x:row>
     <x:row r="183" ht="24" customHeight="1">
       <x:c r="A183" s="19"/>
@@ -2087,6 +2341,7 @@
       <x:c r="E183" s="17"/>
       <x:c r="F183" s="17"/>
       <x:c r="G183" s="17"/>
+      <x:c r="H183" s="42"/>
     </x:row>
     <x:row r="184" ht="24" customHeight="1">
       <x:c r="A184" s="19"/>
@@ -2096,6 +2351,7 @@
       <x:c r="E184" s="17"/>
       <x:c r="F184" s="17"/>
       <x:c r="G184" s="17"/>
+      <x:c r="H184" s="42"/>
     </x:row>
     <x:row r="185" ht="24" customHeight="1">
       <x:c r="A185" s="19"/>
@@ -2105,6 +2361,7 @@
       <x:c r="E185" s="17"/>
       <x:c r="F185" s="17"/>
       <x:c r="G185" s="17"/>
+      <x:c r="H185" s="42"/>
     </x:row>
     <x:row r="186" ht="24" customHeight="1">
       <x:c r="A186" s="19"/>
@@ -2114,6 +2371,7 @@
       <x:c r="E186" s="17"/>
       <x:c r="F186" s="17"/>
       <x:c r="G186" s="17"/>
+      <x:c r="H186" s="42"/>
     </x:row>
     <x:row r="187" ht="24" customHeight="1">
       <x:c r="A187" s="19"/>
@@ -2123,6 +2381,7 @@
       <x:c r="E187" s="17"/>
       <x:c r="F187" s="17"/>
       <x:c r="G187" s="17"/>
+      <x:c r="H187" s="42"/>
     </x:row>
     <x:row r="188" ht="24" customHeight="1">
       <x:c r="A188" s="19"/>
@@ -2132,6 +2391,7 @@
       <x:c r="E188" s="17"/>
       <x:c r="F188" s="17"/>
       <x:c r="G188" s="17"/>
+      <x:c r="H188" s="42"/>
     </x:row>
     <x:row r="189" ht="24" customHeight="1">
       <x:c r="A189" s="19"/>
@@ -2141,6 +2401,7 @@
       <x:c r="E189" s="17"/>
       <x:c r="F189" s="17"/>
       <x:c r="G189" s="17"/>
+      <x:c r="H189" s="42"/>
     </x:row>
     <x:row r="190" ht="24" customHeight="1">
       <x:c r="A190" s="19"/>
@@ -2150,6 +2411,7 @@
       <x:c r="E190" s="17"/>
       <x:c r="F190" s="17"/>
       <x:c r="G190" s="17"/>
+      <x:c r="H190" s="42"/>
     </x:row>
     <x:row r="191" ht="24" customHeight="1">
       <x:c r="A191" s="19"/>
@@ -2159,6 +2421,7 @@
       <x:c r="E191" s="17"/>
       <x:c r="F191" s="17"/>
       <x:c r="G191" s="17"/>
+      <x:c r="H191" s="42"/>
     </x:row>
     <x:row r="192" ht="24" customHeight="1">
       <x:c r="A192" s="19"/>
@@ -2168,6 +2431,7 @@
       <x:c r="E192" s="17"/>
       <x:c r="F192" s="17"/>
       <x:c r="G192" s="17"/>
+      <x:c r="H192" s="42"/>
     </x:row>
     <x:row r="193" ht="24" customHeight="1">
       <x:c r="A193" s="19"/>
@@ -2177,6 +2441,7 @@
       <x:c r="E193" s="17"/>
       <x:c r="F193" s="17"/>
       <x:c r="G193" s="17"/>
+      <x:c r="H193" s="42"/>
     </x:row>
     <x:row r="194" ht="24" customHeight="1">
       <x:c r="A194" s="19"/>
@@ -2186,6 +2451,7 @@
       <x:c r="E194" s="17"/>
       <x:c r="F194" s="17"/>
       <x:c r="G194" s="17"/>
+      <x:c r="H194" s="42"/>
     </x:row>
     <x:row r="195" ht="24" customHeight="1">
       <x:c r="A195" s="19"/>
@@ -2195,6 +2461,7 @@
       <x:c r="E195" s="17"/>
       <x:c r="F195" s="17"/>
       <x:c r="G195" s="17"/>
+      <x:c r="H195" s="42"/>
     </x:row>
     <x:row r="196" ht="24" customHeight="1">
       <x:c r="A196" s="19"/>
@@ -2204,6 +2471,7 @@
       <x:c r="E196" s="17"/>
       <x:c r="F196" s="17"/>
       <x:c r="G196" s="17"/>
+      <x:c r="H196" s="42"/>
     </x:row>
     <x:row r="197" ht="24" customHeight="1">
       <x:c r="A197" s="19"/>
@@ -2213,6 +2481,7 @@
       <x:c r="E197" s="17"/>
       <x:c r="F197" s="17"/>
       <x:c r="G197" s="17"/>
+      <x:c r="H197" s="42"/>
     </x:row>
     <x:row r="198" ht="24" customHeight="1">
       <x:c r="A198" s="19"/>
@@ -2222,6 +2491,7 @@
       <x:c r="E198" s="17"/>
       <x:c r="F198" s="17"/>
       <x:c r="G198" s="17"/>
+      <x:c r="H198" s="42"/>
     </x:row>
     <x:row r="199" ht="24" customHeight="1">
       <x:c r="A199" s="19"/>
@@ -2231,6 +2501,7 @@
       <x:c r="E199" s="17"/>
       <x:c r="F199" s="17"/>
       <x:c r="G199" s="17"/>
+      <x:c r="H199" s="42"/>
     </x:row>
     <x:row r="200" ht="24" customHeight="1">
       <x:c r="A200" s="19"/>
@@ -2240,6 +2511,7 @@
       <x:c r="E200" s="17"/>
       <x:c r="F200" s="17"/>
       <x:c r="G200" s="17"/>
+      <x:c r="H200" s="42"/>
     </x:row>
     <x:row r="201" ht="24" customHeight="1">
       <x:c r="A201" s="19"/>
@@ -2249,6 +2521,904 @@
       <x:c r="E201" s="17"/>
       <x:c r="F201" s="17"/>
       <x:c r="G201" s="17"/>
+      <x:c r="H201" s="42"/>
+    </x:row>
+    <x:row r="202" ht="24" customHeight="1">
+      <x:c r="H202" s="42"/>
+    </x:row>
+    <x:row r="203" ht="24" customHeight="1">
+      <x:c r="H203" s="42"/>
+    </x:row>
+    <x:row r="204" ht="24" customHeight="1">
+      <x:c r="H204" s="42"/>
+    </x:row>
+    <x:row r="205" ht="24" customHeight="1">
+      <x:c r="H205" s="42"/>
+    </x:row>
+    <x:row r="206" ht="24" customHeight="1">
+      <x:c r="H206" s="42"/>
+    </x:row>
+    <x:row r="207" ht="24" customHeight="1">
+      <x:c r="H207" s="42"/>
+    </x:row>
+    <x:row r="208" ht="24" customHeight="1">
+      <x:c r="H208" s="42"/>
+    </x:row>
+    <x:row r="209" ht="24" customHeight="1">
+      <x:c r="H209" s="42"/>
+    </x:row>
+    <x:row r="210" ht="24" customHeight="1">
+      <x:c r="H210" s="42"/>
+    </x:row>
+    <x:row r="211" ht="24" customHeight="1">
+      <x:c r="H211" s="42"/>
+    </x:row>
+    <x:row r="212" ht="24" customHeight="1">
+      <x:c r="H212" s="42"/>
+    </x:row>
+    <x:row r="213" ht="24" customHeight="1">
+      <x:c r="H213" s="42"/>
+    </x:row>
+    <x:row r="214" ht="24" customHeight="1">
+      <x:c r="H214" s="42"/>
+    </x:row>
+    <x:row r="215" ht="24" customHeight="1">
+      <x:c r="H215" s="42"/>
+    </x:row>
+    <x:row r="216" ht="24" customHeight="1">
+      <x:c r="H216" s="42"/>
+    </x:row>
+    <x:row r="217" ht="24" customHeight="1">
+      <x:c r="H217" s="42"/>
+    </x:row>
+    <x:row r="218" ht="24" customHeight="1">
+      <x:c r="H218" s="42"/>
+    </x:row>
+    <x:row r="219" ht="24" customHeight="1">
+      <x:c r="H219" s="42"/>
+    </x:row>
+    <x:row r="220" ht="24" customHeight="1">
+      <x:c r="H220" s="42"/>
+    </x:row>
+    <x:row r="221" ht="24" customHeight="1">
+      <x:c r="H221" s="42"/>
+    </x:row>
+    <x:row r="222" ht="24" customHeight="1">
+      <x:c r="H222" s="42"/>
+    </x:row>
+    <x:row r="223" ht="24" customHeight="1">
+      <x:c r="H223" s="42"/>
+    </x:row>
+    <x:row r="224" ht="24" customHeight="1">
+      <x:c r="H224" s="42"/>
+    </x:row>
+    <x:row r="225" ht="24" customHeight="1">
+      <x:c r="H225" s="42"/>
+    </x:row>
+    <x:row r="226" ht="24" customHeight="1">
+      <x:c r="H226" s="42"/>
+    </x:row>
+    <x:row r="227" ht="24" customHeight="1">
+      <x:c r="H227" s="42"/>
+    </x:row>
+    <x:row r="228" ht="24" customHeight="1">
+      <x:c r="H228" s="42"/>
+    </x:row>
+    <x:row r="229" ht="24" customHeight="1">
+      <x:c r="H229" s="42"/>
+    </x:row>
+    <x:row r="230" ht="24" customHeight="1">
+      <x:c r="H230" s="42"/>
+    </x:row>
+    <x:row r="231" ht="24" customHeight="1">
+      <x:c r="H231" s="42"/>
+    </x:row>
+    <x:row r="232" ht="24" customHeight="1">
+      <x:c r="H232" s="42"/>
+    </x:row>
+    <x:row r="233" ht="24" customHeight="1">
+      <x:c r="H233" s="42"/>
+    </x:row>
+    <x:row r="234" ht="24" customHeight="1">
+      <x:c r="H234" s="42"/>
+    </x:row>
+    <x:row r="235" ht="24" customHeight="1">
+      <x:c r="H235" s="42"/>
+    </x:row>
+    <x:row r="236" ht="24" customHeight="1">
+      <x:c r="H236" s="42"/>
+    </x:row>
+    <x:row r="237" ht="24" customHeight="1">
+      <x:c r="H237" s="42"/>
+    </x:row>
+    <x:row r="238" ht="24" customHeight="1">
+      <x:c r="H238" s="42"/>
+    </x:row>
+    <x:row r="239" ht="24" customHeight="1">
+      <x:c r="H239" s="42"/>
+    </x:row>
+    <x:row r="240" ht="24" customHeight="1">
+      <x:c r="H240" s="42"/>
+    </x:row>
+    <x:row r="241" ht="24" customHeight="1">
+      <x:c r="H241" s="42"/>
+    </x:row>
+    <x:row r="242" ht="24" customHeight="1">
+      <x:c r="H242" s="42"/>
+    </x:row>
+    <x:row r="243" ht="24" customHeight="1">
+      <x:c r="H243" s="42"/>
+    </x:row>
+    <x:row r="244" ht="24" customHeight="1">
+      <x:c r="H244" s="42"/>
+    </x:row>
+    <x:row r="245" ht="24" customHeight="1">
+      <x:c r="H245" s="42"/>
+    </x:row>
+    <x:row r="246" ht="24" customHeight="1">
+      <x:c r="H246" s="42"/>
+    </x:row>
+    <x:row r="247" ht="24" customHeight="1">
+      <x:c r="H247" s="42"/>
+    </x:row>
+    <x:row r="248" ht="24" customHeight="1">
+      <x:c r="H248" s="42"/>
+    </x:row>
+    <x:row r="249" ht="24" customHeight="1">
+      <x:c r="H249" s="42"/>
+    </x:row>
+    <x:row r="250" ht="24" customHeight="1">
+      <x:c r="H250" s="42"/>
+    </x:row>
+    <x:row r="251" ht="24" customHeight="1">
+      <x:c r="H251" s="42"/>
+    </x:row>
+    <x:row r="252" ht="24" customHeight="1">
+      <x:c r="H252" s="42"/>
+    </x:row>
+    <x:row r="253" ht="24" customHeight="1">
+      <x:c r="H253" s="42"/>
+    </x:row>
+    <x:row r="254" ht="24" customHeight="1">
+      <x:c r="H254" s="42"/>
+    </x:row>
+    <x:row r="255" ht="24" customHeight="1">
+      <x:c r="H255" s="42"/>
+    </x:row>
+    <x:row r="256" ht="24" customHeight="1">
+      <x:c r="H256" s="42"/>
+    </x:row>
+    <x:row r="257" ht="24" customHeight="1">
+      <x:c r="H257" s="42"/>
+    </x:row>
+    <x:row r="258" ht="24" customHeight="1">
+      <x:c r="H258" s="42"/>
+    </x:row>
+    <x:row r="259" ht="24" customHeight="1">
+      <x:c r="H259" s="42"/>
+    </x:row>
+    <x:row r="260" ht="24" customHeight="1">
+      <x:c r="H260" s="42"/>
+    </x:row>
+    <x:row r="261" ht="24" customHeight="1">
+      <x:c r="H261" s="42"/>
+    </x:row>
+    <x:row r="262" ht="24" customHeight="1">
+      <x:c r="H262" s="42"/>
+    </x:row>
+    <x:row r="263" ht="24" customHeight="1">
+      <x:c r="H263" s="42"/>
+    </x:row>
+    <x:row r="264" ht="24" customHeight="1">
+      <x:c r="H264" s="42"/>
+    </x:row>
+    <x:row r="265" ht="24" customHeight="1">
+      <x:c r="H265" s="42"/>
+    </x:row>
+    <x:row r="266" ht="24" customHeight="1">
+      <x:c r="H266" s="42"/>
+    </x:row>
+    <x:row r="267" ht="24" customHeight="1">
+      <x:c r="H267" s="42"/>
+    </x:row>
+    <x:row r="268" ht="24" customHeight="1">
+      <x:c r="H268" s="42"/>
+    </x:row>
+    <x:row r="269" ht="24" customHeight="1">
+      <x:c r="H269" s="42"/>
+    </x:row>
+    <x:row r="270" ht="24" customHeight="1">
+      <x:c r="H270" s="42"/>
+    </x:row>
+    <x:row r="271" ht="24" customHeight="1">
+      <x:c r="H271" s="42"/>
+    </x:row>
+    <x:row r="272" ht="24" customHeight="1">
+      <x:c r="H272" s="42"/>
+    </x:row>
+    <x:row r="273" ht="24" customHeight="1">
+      <x:c r="H273" s="42"/>
+    </x:row>
+    <x:row r="274" ht="24" customHeight="1">
+      <x:c r="H274" s="42"/>
+    </x:row>
+    <x:row r="275" ht="24" customHeight="1">
+      <x:c r="H275" s="42"/>
+    </x:row>
+    <x:row r="276" ht="24" customHeight="1">
+      <x:c r="H276" s="42"/>
+    </x:row>
+    <x:row r="277" ht="24" customHeight="1">
+      <x:c r="H277" s="42"/>
+    </x:row>
+    <x:row r="278" ht="24" customHeight="1">
+      <x:c r="H278" s="42"/>
+    </x:row>
+    <x:row r="279" ht="24" customHeight="1">
+      <x:c r="H279" s="42"/>
+    </x:row>
+    <x:row r="280" ht="24" customHeight="1">
+      <x:c r="H280" s="42"/>
+    </x:row>
+    <x:row r="281" ht="24" customHeight="1">
+      <x:c r="H281" s="42"/>
+    </x:row>
+    <x:row r="282" ht="24" customHeight="1">
+      <x:c r="H282" s="42"/>
+    </x:row>
+    <x:row r="283" ht="24" customHeight="1">
+      <x:c r="H283" s="42"/>
+    </x:row>
+    <x:row r="284" ht="24" customHeight="1">
+      <x:c r="H284" s="42"/>
+    </x:row>
+    <x:row r="285" ht="24" customHeight="1">
+      <x:c r="H285" s="42"/>
+    </x:row>
+    <x:row r="286" ht="24" customHeight="1">
+      <x:c r="H286" s="42"/>
+    </x:row>
+    <x:row r="287" ht="24" customHeight="1">
+      <x:c r="H287" s="42"/>
+    </x:row>
+    <x:row r="288" ht="24" customHeight="1">
+      <x:c r="H288" s="42"/>
+    </x:row>
+    <x:row r="289" ht="24" customHeight="1">
+      <x:c r="H289" s="42"/>
+    </x:row>
+    <x:row r="290" ht="24" customHeight="1">
+      <x:c r="H290" s="42"/>
+    </x:row>
+    <x:row r="291" ht="24" customHeight="1">
+      <x:c r="H291" s="42"/>
+    </x:row>
+    <x:row r="292" ht="24" customHeight="1">
+      <x:c r="H292" s="42"/>
+    </x:row>
+    <x:row r="293" ht="24" customHeight="1">
+      <x:c r="H293" s="42"/>
+    </x:row>
+    <x:row r="294" ht="24" customHeight="1">
+      <x:c r="H294" s="42"/>
+    </x:row>
+    <x:row r="295" ht="24" customHeight="1">
+      <x:c r="H295" s="42"/>
+    </x:row>
+    <x:row r="296" ht="24" customHeight="1">
+      <x:c r="H296" s="42"/>
+    </x:row>
+    <x:row r="297" ht="24" customHeight="1">
+      <x:c r="H297" s="42"/>
+    </x:row>
+    <x:row r="298" ht="24" customHeight="1">
+      <x:c r="H298" s="42"/>
+    </x:row>
+    <x:row r="299" ht="24" customHeight="1">
+      <x:c r="H299" s="42"/>
+    </x:row>
+    <x:row r="300" ht="24" customHeight="1">
+      <x:c r="H300" s="42"/>
+    </x:row>
+    <x:row r="301" ht="24" customHeight="1">
+      <x:c r="H301" s="42"/>
+    </x:row>
+    <x:row r="302" ht="24" customHeight="1">
+      <x:c r="H302" s="42"/>
+    </x:row>
+    <x:row r="303" ht="24" customHeight="1">
+      <x:c r="H303" s="42"/>
+    </x:row>
+    <x:row r="304" ht="24" customHeight="1">
+      <x:c r="H304" s="42"/>
+    </x:row>
+    <x:row r="305" ht="24" customHeight="1">
+      <x:c r="H305" s="42"/>
+    </x:row>
+    <x:row r="306" ht="24" customHeight="1">
+      <x:c r="H306" s="42"/>
+    </x:row>
+    <x:row r="307" ht="24" customHeight="1">
+      <x:c r="H307" s="42"/>
+    </x:row>
+    <x:row r="308" ht="24" customHeight="1">
+      <x:c r="H308" s="42"/>
+    </x:row>
+    <x:row r="309" ht="24" customHeight="1">
+      <x:c r="H309" s="42"/>
+    </x:row>
+    <x:row r="310" ht="24" customHeight="1">
+      <x:c r="H310" s="42"/>
+    </x:row>
+    <x:row r="311" ht="24" customHeight="1">
+      <x:c r="H311" s="42"/>
+    </x:row>
+    <x:row r="312" ht="24" customHeight="1">
+      <x:c r="H312" s="42"/>
+    </x:row>
+    <x:row r="313" ht="24" customHeight="1">
+      <x:c r="H313" s="42"/>
+    </x:row>
+    <x:row r="314" ht="24" customHeight="1">
+      <x:c r="H314" s="42"/>
+    </x:row>
+    <x:row r="315" ht="24" customHeight="1">
+      <x:c r="H315" s="42"/>
+    </x:row>
+    <x:row r="316" ht="24" customHeight="1">
+      <x:c r="H316" s="42"/>
+    </x:row>
+    <x:row r="317" ht="24" customHeight="1">
+      <x:c r="H317" s="42"/>
+    </x:row>
+    <x:row r="318" ht="24" customHeight="1">
+      <x:c r="H318" s="42"/>
+    </x:row>
+    <x:row r="319" ht="24" customHeight="1">
+      <x:c r="H319" s="42"/>
+    </x:row>
+    <x:row r="320" ht="24" customHeight="1">
+      <x:c r="H320" s="42"/>
+    </x:row>
+    <x:row r="321" ht="24" customHeight="1">
+      <x:c r="H321" s="42"/>
+    </x:row>
+    <x:row r="322" ht="24" customHeight="1">
+      <x:c r="H322" s="42"/>
+    </x:row>
+    <x:row r="323" ht="24" customHeight="1">
+      <x:c r="H323" s="42"/>
+    </x:row>
+    <x:row r="324" ht="24" customHeight="1">
+      <x:c r="H324" s="42"/>
+    </x:row>
+    <x:row r="325" ht="24" customHeight="1">
+      <x:c r="H325" s="42"/>
+    </x:row>
+    <x:row r="326" ht="24" customHeight="1">
+      <x:c r="H326" s="42"/>
+    </x:row>
+    <x:row r="327" ht="24" customHeight="1">
+      <x:c r="H327" s="42"/>
+    </x:row>
+    <x:row r="328" ht="24" customHeight="1">
+      <x:c r="H328" s="42"/>
+    </x:row>
+    <x:row r="329" ht="24" customHeight="1">
+      <x:c r="H329" s="42"/>
+    </x:row>
+    <x:row r="330" ht="24" customHeight="1">
+      <x:c r="H330" s="42"/>
+    </x:row>
+    <x:row r="331" ht="24" customHeight="1">
+      <x:c r="H331" s="42"/>
+    </x:row>
+    <x:row r="332" ht="24" customHeight="1">
+      <x:c r="H332" s="42"/>
+    </x:row>
+    <x:row r="333" ht="24" customHeight="1">
+      <x:c r="H333" s="42"/>
+    </x:row>
+    <x:row r="334" ht="24" customHeight="1">
+      <x:c r="H334" s="42"/>
+    </x:row>
+    <x:row r="335" ht="24" customHeight="1">
+      <x:c r="H335" s="42"/>
+    </x:row>
+    <x:row r="336" ht="24" customHeight="1">
+      <x:c r="H336" s="42"/>
+    </x:row>
+    <x:row r="337" ht="24" customHeight="1">
+      <x:c r="H337" s="42"/>
+    </x:row>
+    <x:row r="338" ht="24" customHeight="1">
+      <x:c r="H338" s="42"/>
+    </x:row>
+    <x:row r="339" ht="24" customHeight="1">
+      <x:c r="H339" s="42"/>
+    </x:row>
+    <x:row r="340" ht="24" customHeight="1">
+      <x:c r="H340" s="42"/>
+    </x:row>
+    <x:row r="341" ht="24" customHeight="1">
+      <x:c r="H341" s="42"/>
+    </x:row>
+    <x:row r="342" ht="24" customHeight="1">
+      <x:c r="H342" s="42"/>
+    </x:row>
+    <x:row r="343" ht="24" customHeight="1">
+      <x:c r="H343" s="42"/>
+    </x:row>
+    <x:row r="344" ht="24" customHeight="1">
+      <x:c r="H344" s="42"/>
+    </x:row>
+    <x:row r="345" ht="24" customHeight="1">
+      <x:c r="H345" s="42"/>
+    </x:row>
+    <x:row r="346" ht="24" customHeight="1">
+      <x:c r="H346" s="42"/>
+    </x:row>
+    <x:row r="347" ht="24" customHeight="1">
+      <x:c r="H347" s="42"/>
+    </x:row>
+    <x:row r="348" ht="24" customHeight="1">
+      <x:c r="H348" s="42"/>
+    </x:row>
+    <x:row r="349" ht="24" customHeight="1">
+      <x:c r="H349" s="42"/>
+    </x:row>
+    <x:row r="350" ht="24" customHeight="1">
+      <x:c r="H350" s="42"/>
+    </x:row>
+    <x:row r="351" ht="24" customHeight="1">
+      <x:c r="H351" s="42"/>
+    </x:row>
+    <x:row r="352" ht="24" customHeight="1">
+      <x:c r="H352" s="42"/>
+    </x:row>
+    <x:row r="353" ht="24" customHeight="1">
+      <x:c r="H353" s="42"/>
+    </x:row>
+    <x:row r="354" ht="24" customHeight="1">
+      <x:c r="H354" s="42"/>
+    </x:row>
+    <x:row r="355" ht="24" customHeight="1">
+      <x:c r="H355" s="42"/>
+    </x:row>
+    <x:row r="356" ht="24" customHeight="1">
+      <x:c r="H356" s="42"/>
+    </x:row>
+    <x:row r="357" ht="24" customHeight="1">
+      <x:c r="H357" s="42"/>
+    </x:row>
+    <x:row r="358" ht="24" customHeight="1">
+      <x:c r="H358" s="42"/>
+    </x:row>
+    <x:row r="359" ht="24" customHeight="1">
+      <x:c r="H359" s="42"/>
+    </x:row>
+    <x:row r="360" ht="24" customHeight="1">
+      <x:c r="H360" s="42"/>
+    </x:row>
+    <x:row r="361" ht="24" customHeight="1">
+      <x:c r="H361" s="42"/>
+    </x:row>
+    <x:row r="362" ht="24" customHeight="1">
+      <x:c r="H362" s="42"/>
+    </x:row>
+    <x:row r="363" ht="24" customHeight="1">
+      <x:c r="H363" s="42"/>
+    </x:row>
+    <x:row r="364" ht="24" customHeight="1">
+      <x:c r="H364" s="42"/>
+    </x:row>
+    <x:row r="365" ht="24" customHeight="1">
+      <x:c r="H365" s="42"/>
+    </x:row>
+    <x:row r="366" ht="24" customHeight="1">
+      <x:c r="H366" s="42"/>
+    </x:row>
+    <x:row r="367" ht="24" customHeight="1">
+      <x:c r="H367" s="42"/>
+    </x:row>
+    <x:row r="368" ht="24" customHeight="1">
+      <x:c r="H368" s="42"/>
+    </x:row>
+    <x:row r="369" ht="24" customHeight="1">
+      <x:c r="H369" s="42"/>
+    </x:row>
+    <x:row r="370" ht="24" customHeight="1">
+      <x:c r="H370" s="42"/>
+    </x:row>
+    <x:row r="371" ht="24" customHeight="1">
+      <x:c r="H371" s="42"/>
+    </x:row>
+    <x:row r="372" ht="24" customHeight="1">
+      <x:c r="H372" s="42"/>
+    </x:row>
+    <x:row r="373" ht="24" customHeight="1">
+      <x:c r="H373" s="42"/>
+    </x:row>
+    <x:row r="374" ht="24" customHeight="1">
+      <x:c r="H374" s="42"/>
+    </x:row>
+    <x:row r="375" ht="24" customHeight="1">
+      <x:c r="H375" s="42"/>
+    </x:row>
+    <x:row r="376" ht="24" customHeight="1">
+      <x:c r="H376" s="42"/>
+    </x:row>
+    <x:row r="377" ht="24" customHeight="1">
+      <x:c r="H377" s="42"/>
+    </x:row>
+    <x:row r="378" ht="24" customHeight="1">
+      <x:c r="H378" s="42"/>
+    </x:row>
+    <x:row r="379" ht="24" customHeight="1">
+      <x:c r="H379" s="42"/>
+    </x:row>
+    <x:row r="380" ht="24" customHeight="1">
+      <x:c r="H380" s="42"/>
+    </x:row>
+    <x:row r="381" ht="24" customHeight="1">
+      <x:c r="H381" s="42"/>
+    </x:row>
+    <x:row r="382" ht="24" customHeight="1">
+      <x:c r="H382" s="42"/>
+    </x:row>
+    <x:row r="383" ht="24" customHeight="1">
+      <x:c r="H383" s="42"/>
+    </x:row>
+    <x:row r="384" ht="24" customHeight="1">
+      <x:c r="H384" s="42"/>
+    </x:row>
+    <x:row r="385" ht="24" customHeight="1">
+      <x:c r="H385" s="42"/>
+    </x:row>
+    <x:row r="386" ht="24" customHeight="1">
+      <x:c r="H386" s="42"/>
+    </x:row>
+    <x:row r="387" ht="24" customHeight="1">
+      <x:c r="H387" s="42"/>
+    </x:row>
+    <x:row r="388" ht="24" customHeight="1">
+      <x:c r="H388" s="42"/>
+    </x:row>
+    <x:row r="389" ht="24" customHeight="1">
+      <x:c r="H389" s="42"/>
+    </x:row>
+    <x:row r="390" ht="24" customHeight="1">
+      <x:c r="H390" s="42"/>
+    </x:row>
+    <x:row r="391" ht="24" customHeight="1">
+      <x:c r="H391" s="42"/>
+    </x:row>
+    <x:row r="392" ht="24" customHeight="1">
+      <x:c r="H392" s="42"/>
+    </x:row>
+    <x:row r="393" ht="24" customHeight="1">
+      <x:c r="H393" s="42"/>
+    </x:row>
+    <x:row r="394" ht="24" customHeight="1">
+      <x:c r="H394" s="42"/>
+    </x:row>
+    <x:row r="395" ht="24" customHeight="1">
+      <x:c r="H395" s="42"/>
+    </x:row>
+    <x:row r="396" ht="24" customHeight="1">
+      <x:c r="H396" s="42"/>
+    </x:row>
+    <x:row r="397" ht="24" customHeight="1">
+      <x:c r="H397" s="42"/>
+    </x:row>
+    <x:row r="398" ht="24" customHeight="1">
+      <x:c r="H398" s="42"/>
+    </x:row>
+    <x:row r="399" ht="24" customHeight="1">
+      <x:c r="H399" s="42"/>
+    </x:row>
+    <x:row r="400" ht="24" customHeight="1">
+      <x:c r="H400" s="42"/>
+    </x:row>
+    <x:row r="401" ht="24" customHeight="1">
+      <x:c r="H401" s="42"/>
+    </x:row>
+    <x:row r="402" ht="24" customHeight="1">
+      <x:c r="H402" s="42"/>
+    </x:row>
+    <x:row r="403" ht="24" customHeight="1">
+      <x:c r="H403" s="42"/>
+    </x:row>
+    <x:row r="404" ht="24" customHeight="1">
+      <x:c r="H404" s="42"/>
+    </x:row>
+    <x:row r="405" ht="24" customHeight="1">
+      <x:c r="H405" s="42"/>
+    </x:row>
+    <x:row r="406" ht="24" customHeight="1">
+      <x:c r="H406" s="42"/>
+    </x:row>
+    <x:row r="407" ht="24" customHeight="1">
+      <x:c r="H407" s="42"/>
+    </x:row>
+    <x:row r="408" ht="24" customHeight="1">
+      <x:c r="H408" s="42"/>
+    </x:row>
+    <x:row r="409" ht="24" customHeight="1">
+      <x:c r="H409" s="42"/>
+    </x:row>
+    <x:row r="410" ht="24" customHeight="1">
+      <x:c r="H410" s="42"/>
+    </x:row>
+    <x:row r="411" ht="24" customHeight="1">
+      <x:c r="H411" s="42"/>
+    </x:row>
+    <x:row r="412" ht="24" customHeight="1">
+      <x:c r="H412" s="42"/>
+    </x:row>
+    <x:row r="413" ht="24" customHeight="1">
+      <x:c r="H413" s="42"/>
+    </x:row>
+    <x:row r="414" ht="24" customHeight="1">
+      <x:c r="H414" s="42"/>
+    </x:row>
+    <x:row r="415" ht="24" customHeight="1">
+      <x:c r="H415" s="42"/>
+    </x:row>
+    <x:row r="416" ht="24" customHeight="1">
+      <x:c r="H416" s="42"/>
+    </x:row>
+    <x:row r="417" ht="24" customHeight="1">
+      <x:c r="H417" s="42"/>
+    </x:row>
+    <x:row r="418" ht="24" customHeight="1">
+      <x:c r="H418" s="42"/>
+    </x:row>
+    <x:row r="419" ht="24" customHeight="1">
+      <x:c r="H419" s="42"/>
+    </x:row>
+    <x:row r="420" ht="24" customHeight="1">
+      <x:c r="H420" s="42"/>
+    </x:row>
+    <x:row r="421" ht="24" customHeight="1">
+      <x:c r="H421" s="42"/>
+    </x:row>
+    <x:row r="422" ht="24" customHeight="1">
+      <x:c r="H422" s="42"/>
+    </x:row>
+    <x:row r="423" ht="24" customHeight="1">
+      <x:c r="H423" s="42"/>
+    </x:row>
+    <x:row r="424" ht="24" customHeight="1">
+      <x:c r="H424" s="42"/>
+    </x:row>
+    <x:row r="425" ht="24" customHeight="1">
+      <x:c r="H425" s="42"/>
+    </x:row>
+    <x:row r="426" ht="24" customHeight="1">
+      <x:c r="H426" s="42"/>
+    </x:row>
+    <x:row r="427" ht="24" customHeight="1">
+      <x:c r="H427" s="42"/>
+    </x:row>
+    <x:row r="428" ht="24" customHeight="1">
+      <x:c r="H428" s="42"/>
+    </x:row>
+    <x:row r="429" ht="24" customHeight="1">
+      <x:c r="H429" s="42"/>
+    </x:row>
+    <x:row r="430" ht="24" customHeight="1">
+      <x:c r="H430" s="42"/>
+    </x:row>
+    <x:row r="431" ht="24" customHeight="1">
+      <x:c r="H431" s="42"/>
+    </x:row>
+    <x:row r="432" ht="24" customHeight="1">
+      <x:c r="H432" s="42"/>
+    </x:row>
+    <x:row r="433" ht="24" customHeight="1">
+      <x:c r="H433" s="42"/>
+    </x:row>
+    <x:row r="434" ht="24" customHeight="1">
+      <x:c r="H434" s="42"/>
+    </x:row>
+    <x:row r="435" ht="24" customHeight="1">
+      <x:c r="H435" s="42"/>
+    </x:row>
+    <x:row r="436" ht="24" customHeight="1">
+      <x:c r="H436" s="42"/>
+    </x:row>
+    <x:row r="437" ht="24" customHeight="1">
+      <x:c r="H437" s="42"/>
+    </x:row>
+    <x:row r="438" ht="24" customHeight="1">
+      <x:c r="H438" s="42"/>
+    </x:row>
+    <x:row r="439" ht="24" customHeight="1">
+      <x:c r="H439" s="42"/>
+    </x:row>
+    <x:row r="440" ht="24" customHeight="1">
+      <x:c r="H440" s="42"/>
+    </x:row>
+    <x:row r="441" ht="24" customHeight="1">
+      <x:c r="H441" s="42"/>
+    </x:row>
+    <x:row r="442" ht="24" customHeight="1">
+      <x:c r="H442" s="42"/>
+    </x:row>
+    <x:row r="443" ht="24" customHeight="1">
+      <x:c r="H443" s="42"/>
+    </x:row>
+    <x:row r="444" ht="24" customHeight="1">
+      <x:c r="H444" s="42"/>
+    </x:row>
+    <x:row r="445" ht="24" customHeight="1">
+      <x:c r="H445" s="42"/>
+    </x:row>
+    <x:row r="446" ht="24" customHeight="1">
+      <x:c r="H446" s="42"/>
+    </x:row>
+    <x:row r="447" ht="24" customHeight="1">
+      <x:c r="H447" s="42"/>
+    </x:row>
+    <x:row r="448" ht="24" customHeight="1">
+      <x:c r="H448" s="42"/>
+    </x:row>
+    <x:row r="449" ht="24" customHeight="1">
+      <x:c r="H449" s="42"/>
+    </x:row>
+    <x:row r="450" ht="24" customHeight="1">
+      <x:c r="H450" s="42"/>
+    </x:row>
+    <x:row r="451" ht="24" customHeight="1">
+      <x:c r="H451" s="42"/>
+    </x:row>
+    <x:row r="452" ht="24" customHeight="1">
+      <x:c r="H452" s="42"/>
+    </x:row>
+    <x:row r="453" ht="24" customHeight="1">
+      <x:c r="H453" s="42"/>
+    </x:row>
+    <x:row r="454" ht="24" customHeight="1">
+      <x:c r="H454" s="42"/>
+    </x:row>
+    <x:row r="455" ht="24" customHeight="1">
+      <x:c r="H455" s="42"/>
+    </x:row>
+    <x:row r="456" ht="24" customHeight="1">
+      <x:c r="H456" s="42"/>
+    </x:row>
+    <x:row r="457" ht="24" customHeight="1">
+      <x:c r="H457" s="42"/>
+    </x:row>
+    <x:row r="458" ht="24" customHeight="1">
+      <x:c r="H458" s="42"/>
+    </x:row>
+    <x:row r="459" ht="24" customHeight="1">
+      <x:c r="H459" s="42"/>
+    </x:row>
+    <x:row r="460" ht="24" customHeight="1">
+      <x:c r="H460" s="42"/>
+    </x:row>
+    <x:row r="461" ht="24" customHeight="1">
+      <x:c r="H461" s="42"/>
+    </x:row>
+    <x:row r="462" ht="24" customHeight="1">
+      <x:c r="H462" s="42"/>
+    </x:row>
+    <x:row r="463" ht="24" customHeight="1">
+      <x:c r="H463" s="42"/>
+    </x:row>
+    <x:row r="464" ht="24" customHeight="1">
+      <x:c r="H464" s="42"/>
+    </x:row>
+    <x:row r="465" ht="24" customHeight="1">
+      <x:c r="H465" s="42"/>
+    </x:row>
+    <x:row r="466" ht="24" customHeight="1">
+      <x:c r="H466" s="42"/>
+    </x:row>
+    <x:row r="467" ht="24" customHeight="1">
+      <x:c r="H467" s="42"/>
+    </x:row>
+    <x:row r="468" ht="24" customHeight="1">
+      <x:c r="H468" s="42"/>
+    </x:row>
+    <x:row r="469" ht="24" customHeight="1">
+      <x:c r="H469" s="42"/>
+    </x:row>
+    <x:row r="470" ht="24" customHeight="1">
+      <x:c r="H470" s="42"/>
+    </x:row>
+    <x:row r="471" ht="24" customHeight="1">
+      <x:c r="H471" s="42"/>
+    </x:row>
+    <x:row r="472" ht="24" customHeight="1">
+      <x:c r="H472" s="42"/>
+    </x:row>
+    <x:row r="473" ht="24" customHeight="1">
+      <x:c r="H473" s="42"/>
+    </x:row>
+    <x:row r="474" ht="24" customHeight="1">
+      <x:c r="H474" s="42"/>
+    </x:row>
+    <x:row r="475" ht="24" customHeight="1">
+      <x:c r="H475" s="42"/>
+    </x:row>
+    <x:row r="476" ht="24" customHeight="1">
+      <x:c r="H476" s="42"/>
+    </x:row>
+    <x:row r="477" ht="24" customHeight="1">
+      <x:c r="H477" s="42"/>
+    </x:row>
+    <x:row r="478" ht="24" customHeight="1">
+      <x:c r="H478" s="42"/>
+    </x:row>
+    <x:row r="479" ht="24" customHeight="1">
+      <x:c r="H479" s="42"/>
+    </x:row>
+    <x:row r="480" ht="24" customHeight="1">
+      <x:c r="H480" s="42"/>
+    </x:row>
+    <x:row r="481" ht="24" customHeight="1">
+      <x:c r="H481" s="42"/>
+    </x:row>
+    <x:row r="482" ht="24" customHeight="1">
+      <x:c r="H482" s="42"/>
+    </x:row>
+    <x:row r="483" ht="24" customHeight="1">
+      <x:c r="H483" s="42"/>
+    </x:row>
+    <x:row r="484" ht="24" customHeight="1">
+      <x:c r="H484" s="42"/>
+    </x:row>
+    <x:row r="485" ht="24" customHeight="1">
+      <x:c r="H485" s="42"/>
+    </x:row>
+    <x:row r="486" ht="24" customHeight="1">
+      <x:c r="H486" s="42"/>
+    </x:row>
+    <x:row r="487" ht="24" customHeight="1">
+      <x:c r="H487" s="42"/>
+    </x:row>
+    <x:row r="488" ht="24" customHeight="1">
+      <x:c r="H488" s="42"/>
+    </x:row>
+    <x:row r="489" ht="24" customHeight="1">
+      <x:c r="H489" s="42"/>
+    </x:row>
+    <x:row r="490" ht="24" customHeight="1">
+      <x:c r="H490" s="42"/>
+    </x:row>
+    <x:row r="491" ht="24" customHeight="1">
+      <x:c r="H491" s="42"/>
+    </x:row>
+    <x:row r="492" ht="24" customHeight="1">
+      <x:c r="H492" s="42"/>
+    </x:row>
+    <x:row r="493" ht="24" customHeight="1">
+      <x:c r="H493" s="42"/>
+    </x:row>
+    <x:row r="494" ht="24" customHeight="1">
+      <x:c r="H494" s="42"/>
+    </x:row>
+    <x:row r="495" ht="24" customHeight="1">
+      <x:c r="H495" s="42"/>
+    </x:row>
+    <x:row r="496" ht="24" customHeight="1">
+      <x:c r="H496" s="42"/>
+    </x:row>
+    <x:row r="497" ht="24" customHeight="1">
+      <x:c r="H497" s="42"/>
+    </x:row>
+    <x:row r="498" ht="24" customHeight="1">
+      <x:c r="H498" s="42"/>
+    </x:row>
+    <x:row r="499" ht="24" customHeight="1">
+      <x:c r="H499" s="42"/>
+    </x:row>
+    <x:row r="500" ht="24" customHeight="1">
+      <x:c r="H500" s="42"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -2287,82 +3457,90 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="34" t="str">
+      <x:c r="A4" s="46" t="str">
         <x:v>零件编号</x:v>
       </x:c>
-      <x:c r="B4" s="32" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>必填；建议使用文本格式，最长40个字符。同编号会更新现有零件。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="35" t="str">
+      <x:c r="A5" s="46" t="str">
         <x:v>零件名称</x:v>
       </x:c>
-      <x:c r="B5" s="33" t="str">
+      <x:c r="B5" s="47" t="str">
         <x:v>必填；最长100个字符。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="35" t="str">
+      <x:c r="A6" s="46" t="str">
         <x:v>单件标准工时（小时）</x:v>
       </x:c>
-      <x:c r="B6" s="33" t="str">
+      <x:c r="B6" s="47" t="str">
         <x:v>必填；填写大于0且不超过1000的数字，例如0.25。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="35" t="str">
+      <x:c r="A7" s="46" t="str">
         <x:v>启用状态</x:v>
       </x:c>
-      <x:c r="B7" s="33" t="str">
+      <x:c r="B7" s="47" t="str">
         <x:v>选填；填写启用或停用。新增零件留空时默认启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="35" t="str">
+      <x:c r="A8" s="46" t="str">
         <x:v>零件用途</x:v>
       </x:c>
-      <x:c r="B8" s="33" t="str">
+      <x:c r="B8" s="47" t="str">
         <x:v>选填；填写附件、整机装配或双用途。新增零件留空时默认附件。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="35" t="str">
+      <x:c r="A9" s="46" t="str">
         <x:v>员工1</x:v>
       </x:c>
-      <x:c r="B9" s="33" t="str">
-        <x:v>选填；只能填写一名员工。整机任务优先交给员工1。不存在的员工会自动创建为固定成员。</x:v>
+      <x:c r="B9" s="47" t="str">
+        <x:v>选填；每格一名员工。整机和附件均优先使用员工1的剩余产能。</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A10" s="35" t="str">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="46" t="str">
         <x:v>员工2</x:v>
       </x:c>
-      <x:c r="B10" s="33" t="str">
-        <x:v>选填；只能填写一名员工，且不能与员工1相同。员工1容量不足时承接整机任务；双用途附件只能由员工2完成。</x:v>
+      <x:c r="B10" s="47" t="str">
+        <x:v>选填；员工1无法在任务周期内完成时使用，不能与员工1重复。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="35" t="str">
+      <x:c r="A11" s="46" t="str">
+        <x:v>员工3</x:v>
+      </x:c>
+      <x:c r="B11" s="47" t="str">
+        <x:v>选填；员工1、员工2仍无法完成时使用，不能与前两级重复。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="46" t="str">
         <x:v>旧模板兼容</x:v>
       </x:c>
-      <x:c r="B11" s="33" t="str">
-        <x:v>旧版“员工”列仍可导入，多名员工用顿号分隔；前两名初始化为员工1和员工2，其余技能保留。</x:v>
+      <x:c r="B12" s="47" t="str">
+        <x:v>旧版“员工”列仍可导入；多名员工用顿号分隔，前三名初始化为员工1、员工2、员工3，其余技能保留。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="35" t="str">
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="46" t="str">
         <x:v>导入限制</x:v>
       </x:c>
-      <x:c r="B12" s="33" t="str">
+      <x:c r="B13" s="47" t="str">
         <x:v>只读取第一张工作表；不支持公式；最多5000条；文件不超过5MB。</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="35" t="str">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="46" t="str">
         <x:v>操作顺序</x:v>
       </x:c>
-      <x:c r="B13" s="33" t="str">
+      <x:c r="B14" s="47" t="str">
         <x:v>填写“零件导入”工作表 → 保存 → 软件中选择“导入表格” → 检查预览 → 确认导入。</x:v>
       </x:c>
     </x:row>

</xml_diff>